<commit_message>
Update template ReadMe branding and remove OneDrive instructions
</commit_message>
<xml_diff>
--- a/shared/workbook-template/shay-sett-template.xlsx
+++ b/shared/workbook-template/shay-sett-template.xlsx
@@ -878,128 +878,116 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="22" customWidth="1"/>
-    <x:col min="2" max="2" width="110" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="26" customHeight="1">
-      <x:c r="A1" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Shay Sett workbook</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B1" s="15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Input instructions</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="26" customHeight="1">
-      <x:c r="A2" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Data source</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B2" s="14" t="str">
-        <x:v>Blank input template. No sample business data or transactions. Enter your own values. Currency: MMK.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="26" customHeight="1">
-      <x:c r="A3" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Business</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B3" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Use one authorized business_id in Settings and every transaction row.</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="26" customHeight="1">
-      <x:c r="A4" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Stable IDs</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B4" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Keep IDs when editing. Give new rows unique IDs. Never use formulas for inputs.</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="26" customHeight="1">
-      <x:c r="A5" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Upload</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B5" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Save as .xlsx, then upload in Data Source settings. All required sheet headers must remain.</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="26" customHeight="1">
-      <x:c r="A6" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Missing records</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B6" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Missing rows are retained with a review warning. Upload does not delete history.</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="26" customHeight="1">
-      <x:c r="A7" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">OneDrive</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B7" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Save into OneDrive, wait for cloud sync, then click Sync Now if connected.</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="26" customHeight="1">
-      <x:c r="A8" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Local files</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B8" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Unsynced local Excel edits require re-upload. They are invisible to Microsoft Graph.</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="26" customHeight="1">
-      <x:c r="A9" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Template</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B9" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Keep one Settings row. Add transaction rows below the headers. Amber cells are inputs.</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="44" customHeight="1">
-      <x:c r="A10" s="23" t="str">
-        <x:v>Settings</x:v>
-      </x:c>
-      <x:c r="B10" s="24" t="str">
-        <x:v>Enter business_id, business_name, currency (MMK), opening_date and opening_cash_mmk before importing. A blank amount is unknown, not zero.</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
+<s:worksheet xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <s:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <s:cols>
+    <s:col min="1" max="1" width="22" customWidth="1"/>
+    <s:col min="2" max="2" width="110" customWidth="1"/>
+  </s:cols>
+  <s:sheetData>
+    <s:row r="1" ht="26" customHeight="1">
+      <s:c r="A1" s="15" t="inlineStr">
+        <s:is>
+          <s:t xml:space="preserve">Shay Sett workbook</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B1" s="15" t="inlineStr">
+        <s:is>
+          <s:t xml:space="preserve">Input instructions</s:t>
+        </s:is>
+      </s:c>
+    </s:row>
+    <s:row r="2" ht="26" customHeight="1">
+      <s:c r="A2" s="14" t="inlineStr">
+        <s:is>
+          <s:t xml:space="preserve">Data source</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B2" s="14" t="str">
+        <s:v>Blank input template. No sample business data or transactions. Enter your own values. Currency: MMK.</s:v>
+      </s:c>
+    </s:row>
+    <s:row r="3" ht="26" customHeight="1">
+      <s:c r="A3" s="14" t="inlineStr">
+        <s:is>
+          <s:t xml:space="preserve">Business</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B3" s="14" t="inlineStr">
+        <s:is>
+          <s:t xml:space="preserve">Use one authorized business_id in Settings and every transaction row.</s:t>
+        </s:is>
+      </s:c>
+    </s:row>
+    <s:row r="4" ht="26" customHeight="1">
+      <s:c r="A4" s="14" t="inlineStr">
+        <s:is>
+          <s:t xml:space="preserve">Stable IDs</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B4" s="14" t="inlineStr">
+        <s:is>
+          <s:t xml:space="preserve">Keep IDs when editing. Give new rows unique IDs. Never use formulas for inputs.</s:t>
+        </s:is>
+      </s:c>
+    </s:row>
+    <s:row r="5" ht="26" customHeight="1">
+      <s:c r="A5" s="14" t="inlineStr">
+        <s:is>
+          <s:t xml:space="preserve">Upload</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B5" s="14" t="inlineStr">
+        <s:is>
+          <s:t xml:space="preserve">Save as .xlsx, then upload in Data Source settings. All required sheet headers must remain.</s:t>
+        </s:is>
+      </s:c>
+    </s:row>
+    <s:row r="6" ht="26" customHeight="1">
+      <s:c r="A6" s="14" t="inlineStr">
+        <s:is>
+          <s:t xml:space="preserve">Missing records</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B6" s="14" t="inlineStr">
+        <s:is>
+          <s:t xml:space="preserve">Missing rows are retained with a review warning. Upload does not delete history.</s:t>
+        </s:is>
+      </s:c>
+    </s:row>
+    <s:row r="7" ht="26" customHeight="1">
+      <s:c r="A7" s="14" t="inlineStr">
+        <s:is>
+          <s:t xml:space="preserve">Local files</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B7" s="14" t="inlineStr">
+        <s:is>
+          <s:t xml:space="preserve">Unsynced local Excel edits require re-upload. They are invisible to Microsoft Graph.</s:t>
+        </s:is>
+      </s:c>
+    </s:row>
+    <s:row r="8" ht="26" customHeight="1">
+      <s:c r="A8" s="14" t="inlineStr">
+        <s:is>
+          <s:t xml:space="preserve">Template</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B8" s="14" t="inlineStr">
+        <s:is>
+          <s:t xml:space="preserve">Keep one Settings row. Add transaction rows below the headers. Amber cells are inputs.</s:t>
+        </s:is>
+      </s:c>
+    </s:row>
+    <s:row r="9" ht="44" customHeight="1">
+      <s:c r="A9" s="23" t="str">
+        <s:v>Settings</s:v>
+      </s:c>
+      <s:c r="B9" s="24" t="str">
+        <s:v>Enter business_id, business_name, currency (MMK), opening_date and opening_cash_mmk before importing. A blank amount is unknown, not zero.</s:v>
+      </s:c>
+    </s:row>
+  </s:sheetData>
+  <s:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</s:worksheet>
 </file>
</xml_diff>